<commit_message>
Torivac web: accesibilidad AA, pulido de plantillas, pipeline de enriquecimiento
- a11y: árbol de categorías con botones aria-expanded (sin controles anidados), contrastes AA; axe-core 0 violaciones en las plantillas clave
- UX: hero con subtítulo, iconos en línea, plurales correctos, botón flotante compacto en móvil, tarjetas de categoría
- pipeline: enrich_catalog.py (variantes/voltaje/propuestas desde PDFs verificados), rebuild.sh, build_prices.py, pruebas smoke y smoke-admin

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013NgtfmD27P2Vfa2C4hR1ow
</commit_message>
<xml_diff>
--- a/torivac-web/data/catalog/prices.demo.xlsx
+++ b/torivac-web/data/catalog/prices.demo.xlsx
@@ -566,7 +566,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -625,7 +625,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -743,7 +743,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -802,7 +802,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -847,7 +847,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -906,7 +906,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -965,7 +965,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1083,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -1142,7 +1142,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1260,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -1319,7 +1319,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -1378,7 +1378,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -1437,7 +1437,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -1496,7 +1496,7 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -1555,7 +1555,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -1614,7 +1614,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -1673,7 +1673,7 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -1732,7 +1732,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -1791,7 +1791,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -1850,7 +1850,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -1909,7 +1909,7 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -1968,7 +1968,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -2027,7 +2027,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -2086,7 +2086,7 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -2145,7 +2145,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -2204,7 +2204,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -2263,7 +2263,7 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -2322,7 +2322,7 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -2381,7 +2381,7 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -2440,7 +2440,7 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -2499,7 +2499,7 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -2617,7 +2617,7 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -2676,7 +2676,7 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -2735,7 +2735,7 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -2794,7 +2794,7 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -2853,7 +2853,7 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -2912,7 +2912,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -2971,7 +2971,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -3030,7 +3030,7 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -3089,7 +3089,7 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -3148,7 +3148,7 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -3207,7 +3207,7 @@
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -3266,7 +3266,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -3325,7 +3325,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -3384,7 +3384,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -3443,7 +3443,7 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -3502,7 +3502,7 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -3561,7 +3561,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -3620,7 +3620,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -3679,7 +3679,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -3738,7 +3738,7 @@
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -3797,7 +3797,7 @@
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -3856,7 +3856,7 @@
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -3915,7 +3915,7 @@
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -3974,7 +3974,7 @@
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -4033,7 +4033,7 @@
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -4092,7 +4092,7 @@
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -4151,7 +4151,7 @@
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -4210,7 +4210,7 @@
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -4269,7 +4269,7 @@
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -4328,7 +4328,7 @@
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -4387,7 +4387,7 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -4432,7 +4432,7 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -4491,7 +4491,7 @@
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -4550,7 +4550,7 @@
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -4609,7 +4609,7 @@
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -4668,7 +4668,7 @@
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -4727,7 +4727,7 @@
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -4786,7 +4786,7 @@
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -4845,7 +4845,7 @@
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -4904,7 +4904,7 @@
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -4963,7 +4963,7 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -5022,7 +5022,7 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -5081,7 +5081,7 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -5126,7 +5126,7 @@
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>
@@ -5185,7 +5185,7 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>2026-10-27T23:10:59Z</t>
+          <t>2026-10-27T23:14:07Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Torivac web: fidelidad de contenido (QA), categorías con subcategorías, canónicas y traducciones de categoría
- qa_content.py: compara el texto del demo con el de la web original (productos 99,4 %, páginas 94,4 %)
- categorías: tarjetas de subcategoría con descripción íntegra, traducciones enlazadas por coincidencia de productos
- páginas: ruta real cuando la canónica apunta a otro idioma (contacto EN)
- hallazgos 10 y 11 (aviso legal incompleto, canónicas incoherentes)

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013NgtfmD27P2Vfa2C4hR1ow
</commit_message>
<xml_diff>
--- a/torivac-web/data/catalog/prices.demo.xlsx
+++ b/torivac-web/data/catalog/prices.demo.xlsx
@@ -566,7 +566,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -625,7 +625,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -743,7 +743,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -802,7 +802,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -847,7 +847,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -906,7 +906,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -965,7 +965,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1083,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -1142,7 +1142,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1260,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -1319,7 +1319,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -1378,7 +1378,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -1437,7 +1437,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -1496,7 +1496,7 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -1555,7 +1555,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -1614,7 +1614,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -1673,7 +1673,7 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -1732,7 +1732,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -1791,7 +1791,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -1850,7 +1850,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -1909,7 +1909,7 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -1968,7 +1968,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -2027,7 +2027,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -2086,7 +2086,7 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -2145,7 +2145,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -2204,7 +2204,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -2263,7 +2263,7 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -2322,7 +2322,7 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -2381,7 +2381,7 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -2440,7 +2440,7 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -2499,7 +2499,7 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -2617,7 +2617,7 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -2676,7 +2676,7 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -2735,7 +2735,7 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -2794,7 +2794,7 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -2853,7 +2853,7 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -2912,7 +2912,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -2971,7 +2971,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -3030,7 +3030,7 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -3089,7 +3089,7 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -3148,7 +3148,7 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -3207,7 +3207,7 @@
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -3266,7 +3266,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -3325,7 +3325,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -3384,7 +3384,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -3443,7 +3443,7 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -3502,7 +3502,7 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -3561,7 +3561,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -3620,7 +3620,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -3679,7 +3679,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -3738,7 +3738,7 @@
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -3797,7 +3797,7 @@
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -3856,7 +3856,7 @@
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -3915,7 +3915,7 @@
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -3974,7 +3974,7 @@
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -4033,7 +4033,7 @@
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -4092,7 +4092,7 @@
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -4151,7 +4151,7 @@
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -4210,7 +4210,7 @@
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -4269,7 +4269,7 @@
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -4328,7 +4328,7 @@
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -4387,7 +4387,7 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -4432,7 +4432,7 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -4491,7 +4491,7 @@
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -4550,7 +4550,7 @@
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -4609,7 +4609,7 @@
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -4668,7 +4668,7 @@
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -4727,7 +4727,7 @@
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -4786,7 +4786,7 @@
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -4845,7 +4845,7 @@
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -4904,7 +4904,7 @@
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -4963,7 +4963,7 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -5022,7 +5022,7 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -5081,7 +5081,7 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -5126,7 +5126,7 @@
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>
@@ -5185,7 +5185,7 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>2026-10-27T23:14:07Z</t>
+          <t>2026-10-27T23:22:14Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
torivac: traducciones de categoría según WPML (sondeo de redirecciones, coherente con el árbol) y propuestas de enlaces mal hechos
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013NgtfmD27P2Vfa2C4hR1ow
</commit_message>
<xml_diff>
--- a/torivac-web/data/catalog/prices.demo.xlsx
+++ b/torivac-web/data/catalog/prices.demo.xlsx
@@ -566,7 +566,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -625,7 +625,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -743,7 +743,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -802,7 +802,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -847,7 +847,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -906,7 +906,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -965,7 +965,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1083,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -1142,7 +1142,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1260,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -1319,7 +1319,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -1378,7 +1378,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -1437,7 +1437,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -1496,7 +1496,7 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -1555,7 +1555,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -1614,7 +1614,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -1673,7 +1673,7 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -1732,7 +1732,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -1791,7 +1791,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -1850,7 +1850,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -1909,7 +1909,7 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -1968,7 +1968,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -2027,7 +2027,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -2086,7 +2086,7 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -2145,7 +2145,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -2204,7 +2204,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -2263,7 +2263,7 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -2322,7 +2322,7 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -2381,7 +2381,7 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -2440,7 +2440,7 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -2499,7 +2499,7 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -2617,7 +2617,7 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -2676,7 +2676,7 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -2735,7 +2735,7 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -2794,7 +2794,7 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -2853,7 +2853,7 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -2912,7 +2912,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -2971,7 +2971,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -3030,7 +3030,7 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -3089,7 +3089,7 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -3148,7 +3148,7 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -3207,7 +3207,7 @@
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -3266,7 +3266,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -3325,7 +3325,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -3384,7 +3384,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -3443,7 +3443,7 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -3502,7 +3502,7 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -3561,7 +3561,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -3620,7 +3620,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -3679,7 +3679,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -3738,7 +3738,7 @@
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -3797,7 +3797,7 @@
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -3856,7 +3856,7 @@
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -3915,7 +3915,7 @@
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -3974,7 +3974,7 @@
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -4033,7 +4033,7 @@
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -4092,7 +4092,7 @@
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -4151,7 +4151,7 @@
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -4210,7 +4210,7 @@
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -4269,7 +4269,7 @@
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -4328,7 +4328,7 @@
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -4387,7 +4387,7 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -4432,7 +4432,7 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -4491,7 +4491,7 @@
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -4550,7 +4550,7 @@
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -4609,7 +4609,7 @@
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -4668,7 +4668,7 @@
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -4727,7 +4727,7 @@
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -4786,7 +4786,7 @@
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -4845,7 +4845,7 @@
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -4904,7 +4904,7 @@
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -4963,7 +4963,7 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -5022,7 +5022,7 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -5081,7 +5081,7 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -5126,7 +5126,7 @@
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>
@@ -5185,7 +5185,7 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>2026-10-27T23:22:14Z</t>
+          <t>2026-10-28T07:01:05Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
torivac: control de UX automático (755 páginas × escritorio/móvil), logo circular sin deformar, banner de fondos, enlaces de imagen, palabras largas, propuestas de texto en otro idioma
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013NgtfmD27P2Vfa2C4hR1ow
</commit_message>
<xml_diff>
--- a/torivac-web/data/catalog/prices.demo.xlsx
+++ b/torivac-web/data/catalog/prices.demo.xlsx
@@ -566,7 +566,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -625,7 +625,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -743,7 +743,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -802,7 +802,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -847,7 +847,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -906,7 +906,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -965,7 +965,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1083,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -1142,7 +1142,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1260,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -1319,7 +1319,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -1378,7 +1378,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -1437,7 +1437,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -1496,7 +1496,7 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -1555,7 +1555,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -1614,7 +1614,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -1673,7 +1673,7 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -1732,7 +1732,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -1791,7 +1791,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -1850,7 +1850,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -1909,7 +1909,7 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -1968,7 +1968,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -2027,7 +2027,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -2086,7 +2086,7 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -2145,7 +2145,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -2204,7 +2204,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -2263,7 +2263,7 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -2322,7 +2322,7 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -2381,7 +2381,7 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -2440,7 +2440,7 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -2499,7 +2499,7 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -2617,7 +2617,7 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -2676,7 +2676,7 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -2735,7 +2735,7 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -2794,7 +2794,7 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -2853,7 +2853,7 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -2912,7 +2912,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -2971,7 +2971,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -3030,7 +3030,7 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -3089,7 +3089,7 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -3148,7 +3148,7 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -3207,7 +3207,7 @@
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -3266,7 +3266,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -3325,7 +3325,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -3384,7 +3384,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -3443,7 +3443,7 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -3502,7 +3502,7 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -3561,7 +3561,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -3620,7 +3620,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -3679,7 +3679,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -3738,7 +3738,7 @@
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -3797,7 +3797,7 @@
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -3856,7 +3856,7 @@
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -3915,7 +3915,7 @@
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -3974,7 +3974,7 @@
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -4033,7 +4033,7 @@
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -4092,7 +4092,7 @@
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -4151,7 +4151,7 @@
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -4210,7 +4210,7 @@
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -4269,7 +4269,7 @@
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -4328,7 +4328,7 @@
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -4387,7 +4387,7 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -4432,7 +4432,7 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -4491,7 +4491,7 @@
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -4550,7 +4550,7 @@
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -4609,7 +4609,7 @@
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -4668,7 +4668,7 @@
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -4727,7 +4727,7 @@
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -4786,7 +4786,7 @@
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -4845,7 +4845,7 @@
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -4904,7 +4904,7 @@
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -4963,7 +4963,7 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -5022,7 +5022,7 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -5081,7 +5081,7 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -5126,7 +5126,7 @@
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>
@@ -5185,7 +5185,7 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>2026-10-28T07:01:05Z</t>
+          <t>2026-10-28T07:23:34Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
torivac: rendimiento (CSS único + fuentes como archivos en producción: LCP móvil ≤1,4 s), imágenes de categorías en local (demo autónoma), prueba de peticiones externas
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013NgtfmD27P2Vfa2C4hR1ow
</commit_message>
<xml_diff>
--- a/torivac-web/data/catalog/prices.demo.xlsx
+++ b/torivac-web/data/catalog/prices.demo.xlsx
@@ -566,7 +566,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -625,7 +625,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -743,7 +743,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -802,7 +802,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -847,7 +847,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -906,7 +906,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -965,7 +965,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1083,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -1142,7 +1142,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1260,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -1319,7 +1319,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -1378,7 +1378,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -1437,7 +1437,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -1496,7 +1496,7 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -1555,7 +1555,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -1614,7 +1614,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -1673,7 +1673,7 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -1732,7 +1732,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -1791,7 +1791,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -1850,7 +1850,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -1909,7 +1909,7 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -1968,7 +1968,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -2027,7 +2027,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -2086,7 +2086,7 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -2145,7 +2145,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -2204,7 +2204,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -2263,7 +2263,7 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -2322,7 +2322,7 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -2381,7 +2381,7 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -2440,7 +2440,7 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -2499,7 +2499,7 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -2617,7 +2617,7 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -2676,7 +2676,7 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -2735,7 +2735,7 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -2794,7 +2794,7 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -2853,7 +2853,7 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -2912,7 +2912,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -2971,7 +2971,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -3030,7 +3030,7 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -3089,7 +3089,7 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -3148,7 +3148,7 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -3207,7 +3207,7 @@
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -3266,7 +3266,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -3325,7 +3325,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -3384,7 +3384,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -3443,7 +3443,7 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -3502,7 +3502,7 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -3561,7 +3561,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -3620,7 +3620,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -3679,7 +3679,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -3738,7 +3738,7 @@
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -3797,7 +3797,7 @@
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -3856,7 +3856,7 @@
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -3915,7 +3915,7 @@
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -3974,7 +3974,7 @@
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -4033,7 +4033,7 @@
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -4092,7 +4092,7 @@
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -4151,7 +4151,7 @@
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -4210,7 +4210,7 @@
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -4269,7 +4269,7 @@
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -4328,7 +4328,7 @@
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -4387,7 +4387,7 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -4432,7 +4432,7 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -4491,7 +4491,7 @@
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -4550,7 +4550,7 @@
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -4609,7 +4609,7 @@
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -4668,7 +4668,7 @@
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -4727,7 +4727,7 @@
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -4786,7 +4786,7 @@
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -4845,7 +4845,7 @@
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -4904,7 +4904,7 @@
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -4963,7 +4963,7 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -5022,7 +5022,7 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -5081,7 +5081,7 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -5126,7 +5126,7 @@
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>
@@ -5185,7 +5185,7 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>2026-10-28T07:23:34Z</t>
+          <t>2026-10-28T07:27:50Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
torivac: páginas legales (política de cookies en 4 idiomas desde el contenido original + enlace en el pie), propuestas legales para el panel
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013NgtfmD27P2Vfa2C4hR1ow
</commit_message>
<xml_diff>
--- a/torivac-web/data/catalog/prices.demo.xlsx
+++ b/torivac-web/data/catalog/prices.demo.xlsx
@@ -566,7 +566,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -625,7 +625,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -743,7 +743,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -802,7 +802,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -847,7 +847,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -906,7 +906,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -965,7 +965,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1083,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -1142,7 +1142,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1260,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -1319,7 +1319,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -1378,7 +1378,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -1437,7 +1437,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -1496,7 +1496,7 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -1555,7 +1555,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -1614,7 +1614,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -1673,7 +1673,7 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -1732,7 +1732,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -1791,7 +1791,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -1850,7 +1850,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -1909,7 +1909,7 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -1968,7 +1968,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -2027,7 +2027,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -2086,7 +2086,7 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -2145,7 +2145,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -2204,7 +2204,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -2263,7 +2263,7 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -2322,7 +2322,7 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -2381,7 +2381,7 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -2440,7 +2440,7 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -2499,7 +2499,7 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -2617,7 +2617,7 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -2676,7 +2676,7 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -2735,7 +2735,7 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -2794,7 +2794,7 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -2853,7 +2853,7 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -2912,7 +2912,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -2971,7 +2971,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -3030,7 +3030,7 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -3089,7 +3089,7 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -3148,7 +3148,7 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -3207,7 +3207,7 @@
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -3266,7 +3266,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -3325,7 +3325,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -3384,7 +3384,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -3443,7 +3443,7 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -3502,7 +3502,7 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -3561,7 +3561,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -3620,7 +3620,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -3679,7 +3679,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -3738,7 +3738,7 @@
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -3797,7 +3797,7 @@
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -3856,7 +3856,7 @@
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -3915,7 +3915,7 @@
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -3974,7 +3974,7 @@
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -4033,7 +4033,7 @@
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -4092,7 +4092,7 @@
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -4151,7 +4151,7 @@
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -4210,7 +4210,7 @@
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -4269,7 +4269,7 @@
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -4328,7 +4328,7 @@
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -4387,7 +4387,7 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -4432,7 +4432,7 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -4491,7 +4491,7 @@
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -4550,7 +4550,7 @@
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -4609,7 +4609,7 @@
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -4668,7 +4668,7 @@
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -4727,7 +4727,7 @@
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -4786,7 +4786,7 @@
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -4845,7 +4845,7 @@
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -4904,7 +4904,7 @@
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -4963,7 +4963,7 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -5022,7 +5022,7 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -5081,7 +5081,7 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -5126,7 +5126,7 @@
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>
@@ -5185,7 +5185,7 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>2026-10-28T07:27:50Z</t>
+          <t>2026-10-28T07:38:15Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
torivac: destinatarios de pedidos confirmados (info@grupotorivac.com y mzamora@torivac.com), dist/ fuera de git
- meta.json, build_catalog.py y wrangler.toml con los destinatarios confirmados por el cliente; remitente pedidos@grupotorivac.com
- pruebas, helpers, textos del panel y documentación al día
- dist/ (60 MB generados, sin HTML) deja de versionarse; .gitignore protege dist/, data/private/ y *.private.*

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013NgtfmD27P2Vfa2C4hR1ow
</commit_message>
<xml_diff>
--- a/torivac-web/data/catalog/prices.demo.xlsx
+++ b/torivac-web/data/catalog/prices.demo.xlsx
@@ -566,7 +566,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -625,7 +625,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -743,7 +743,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -802,7 +802,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -847,7 +847,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -906,7 +906,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -965,7 +965,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1083,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -1142,7 +1142,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1260,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -1319,7 +1319,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -1378,7 +1378,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -1437,7 +1437,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -1496,7 +1496,7 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -1555,7 +1555,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -1614,7 +1614,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -1673,7 +1673,7 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -1732,7 +1732,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -1791,7 +1791,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -1850,7 +1850,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -1909,7 +1909,7 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -1968,7 +1968,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -2027,7 +2027,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -2086,7 +2086,7 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -2145,7 +2145,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -2204,7 +2204,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -2263,7 +2263,7 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -2322,7 +2322,7 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -2381,7 +2381,7 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -2440,7 +2440,7 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -2499,7 +2499,7 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -2617,7 +2617,7 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -2676,7 +2676,7 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -2735,7 +2735,7 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -2794,7 +2794,7 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -2853,7 +2853,7 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -2912,7 +2912,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -2971,7 +2971,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -3030,7 +3030,7 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -3089,7 +3089,7 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -3148,7 +3148,7 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -3207,7 +3207,7 @@
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -3266,7 +3266,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -3325,7 +3325,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -3384,7 +3384,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -3443,7 +3443,7 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -3502,7 +3502,7 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -3561,7 +3561,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -3620,7 +3620,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -3679,7 +3679,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -3738,7 +3738,7 @@
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -3797,7 +3797,7 @@
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -3856,7 +3856,7 @@
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -3915,7 +3915,7 @@
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -3974,7 +3974,7 @@
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -4033,7 +4033,7 @@
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -4092,7 +4092,7 @@
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -4151,7 +4151,7 @@
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -4210,7 +4210,7 @@
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -4269,7 +4269,7 @@
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -4328,7 +4328,7 @@
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -4387,7 +4387,7 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -4432,7 +4432,7 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -4491,7 +4491,7 @@
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -4550,7 +4550,7 @@
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -4609,7 +4609,7 @@
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -4668,7 +4668,7 @@
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -4727,7 +4727,7 @@
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -4786,7 +4786,7 @@
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -4845,7 +4845,7 @@
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -4904,7 +4904,7 @@
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -4963,7 +4963,7 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -5022,7 +5022,7 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -5081,7 +5081,7 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -5126,7 +5126,7 @@
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>
@@ -5185,7 +5185,7 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>2026-10-28T07:38:15Z</t>
+          <t>2026-10-28T08:20:51Z</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
torivac: demo en un solo archivo por página y aviso si se abre sin estilos
- scripts/single_file.mjs: una página del demo → un .html autosuficiente (CSS, JS, fuentes e imágenes dentro) para verla sin descomprimir nada.
- Demo (sin --base): si la página se abre sin sus hojas de estilo (p. ej. index.html dentro del .zip sin extraer) enseña arriba, en 4 idiomas, cómo abrirla bien.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_013NgtfmD27P2Vfa2C4hR1ow
</commit_message>
<xml_diff>
--- a/torivac-web/data/catalog/prices.demo.xlsx
+++ b/torivac-web/data/catalog/prices.demo.xlsx
@@ -566,7 +566,7 @@
       </c>
       <c r="O2" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -625,7 +625,7 @@
       </c>
       <c r="O3" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -684,7 +684,7 @@
       </c>
       <c r="O4" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -743,7 +743,7 @@
       </c>
       <c r="O5" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -802,7 +802,7 @@
       </c>
       <c r="O6" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -847,7 +847,7 @@
       </c>
       <c r="O7" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -906,7 +906,7 @@
       </c>
       <c r="O8" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -965,7 +965,7 @@
       </c>
       <c r="O9" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -1024,7 +1024,7 @@
       </c>
       <c r="O10" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -1083,7 +1083,7 @@
       </c>
       <c r="O11" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -1142,7 +1142,7 @@
       </c>
       <c r="O12" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -1201,7 +1201,7 @@
       </c>
       <c r="O13" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -1260,7 +1260,7 @@
       </c>
       <c r="O14" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -1319,7 +1319,7 @@
       </c>
       <c r="O15" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -1378,7 +1378,7 @@
       </c>
       <c r="O16" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -1437,7 +1437,7 @@
       </c>
       <c r="O17" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -1496,7 +1496,7 @@
       </c>
       <c r="O18" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -1555,7 +1555,7 @@
       </c>
       <c r="O19" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -1614,7 +1614,7 @@
       </c>
       <c r="O20" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -1673,7 +1673,7 @@
       </c>
       <c r="O21" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -1732,7 +1732,7 @@
       </c>
       <c r="O22" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -1791,7 +1791,7 @@
       </c>
       <c r="O23" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -1850,7 +1850,7 @@
       </c>
       <c r="O24" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -1909,7 +1909,7 @@
       </c>
       <c r="O25" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -1968,7 +1968,7 @@
       </c>
       <c r="O26" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -2027,7 +2027,7 @@
       </c>
       <c r="O27" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -2086,7 +2086,7 @@
       </c>
       <c r="O28" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -2145,7 +2145,7 @@
       </c>
       <c r="O29" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -2204,7 +2204,7 @@
       </c>
       <c r="O30" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -2263,7 +2263,7 @@
       </c>
       <c r="O31" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -2322,7 +2322,7 @@
       </c>
       <c r="O32" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -2381,7 +2381,7 @@
       </c>
       <c r="O33" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -2440,7 +2440,7 @@
       </c>
       <c r="O34" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -2499,7 +2499,7 @@
       </c>
       <c r="O35" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -2558,7 +2558,7 @@
       </c>
       <c r="O36" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -2617,7 +2617,7 @@
       </c>
       <c r="O37" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -2676,7 +2676,7 @@
       </c>
       <c r="O38" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -2735,7 +2735,7 @@
       </c>
       <c r="O39" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -2794,7 +2794,7 @@
       </c>
       <c r="O40" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -2853,7 +2853,7 @@
       </c>
       <c r="O41" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -2912,7 +2912,7 @@
       </c>
       <c r="O42" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -2971,7 +2971,7 @@
       </c>
       <c r="O43" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -3030,7 +3030,7 @@
       </c>
       <c r="O44" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -3089,7 +3089,7 @@
       </c>
       <c r="O45" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -3148,7 +3148,7 @@
       </c>
       <c r="O46" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -3207,7 +3207,7 @@
       </c>
       <c r="O47" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -3266,7 +3266,7 @@
       </c>
       <c r="O48" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -3325,7 +3325,7 @@
       </c>
       <c r="O49" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -3384,7 +3384,7 @@
       </c>
       <c r="O50" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -3443,7 +3443,7 @@
       </c>
       <c r="O51" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -3502,7 +3502,7 @@
       </c>
       <c r="O52" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -3561,7 +3561,7 @@
       </c>
       <c r="O53" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -3620,7 +3620,7 @@
       </c>
       <c r="O54" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -3679,7 +3679,7 @@
       </c>
       <c r="O55" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -3738,7 +3738,7 @@
       </c>
       <c r="O56" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -3797,7 +3797,7 @@
       </c>
       <c r="O57" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -3856,7 +3856,7 @@
       </c>
       <c r="O58" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -3915,7 +3915,7 @@
       </c>
       <c r="O59" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -3974,7 +3974,7 @@
       </c>
       <c r="O60" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -4033,7 +4033,7 @@
       </c>
       <c r="O61" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -4092,7 +4092,7 @@
       </c>
       <c r="O62" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -4151,7 +4151,7 @@
       </c>
       <c r="O63" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -4210,7 +4210,7 @@
       </c>
       <c r="O64" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -4269,7 +4269,7 @@
       </c>
       <c r="O65" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -4328,7 +4328,7 @@
       </c>
       <c r="O66" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -4387,7 +4387,7 @@
       </c>
       <c r="O67" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -4446,7 +4446,7 @@
       </c>
       <c r="O68" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -4505,7 +4505,7 @@
       </c>
       <c r="O69" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -4564,7 +4564,7 @@
       </c>
       <c r="O70" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -4623,7 +4623,7 @@
       </c>
       <c r="O71" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -4682,7 +4682,7 @@
       </c>
       <c r="O72" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -4741,7 +4741,7 @@
       </c>
       <c r="O73" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -4800,7 +4800,7 @@
       </c>
       <c r="O74" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -4859,7 +4859,7 @@
       </c>
       <c r="O75" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -4918,7 +4918,7 @@
       </c>
       <c r="O76" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -4977,7 +4977,7 @@
       </c>
       <c r="O77" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -5036,7 +5036,7 @@
       </c>
       <c r="O78" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -5095,7 +5095,7 @@
       </c>
       <c r="O79" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -5154,7 +5154,7 @@
       </c>
       <c r="O80" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -5213,7 +5213,7 @@
       </c>
       <c r="O81" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -5272,7 +5272,7 @@
       </c>
       <c r="O82" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -5331,7 +5331,7 @@
       </c>
       <c r="O83" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -5390,7 +5390,7 @@
       </c>
       <c r="O84" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -5449,7 +5449,7 @@
       </c>
       <c r="O85" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -5508,7 +5508,7 @@
       </c>
       <c r="O86" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -5567,7 +5567,7 @@
       </c>
       <c r="O87" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -5626,7 +5626,7 @@
       </c>
       <c r="O88" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -5685,7 +5685,7 @@
       </c>
       <c r="O89" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -5744,7 +5744,7 @@
       </c>
       <c r="O90" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -5803,7 +5803,7 @@
       </c>
       <c r="O91" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -5862,7 +5862,7 @@
       </c>
       <c r="O92" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -5921,7 +5921,7 @@
       </c>
       <c r="O93" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -5980,7 +5980,7 @@
       </c>
       <c r="O94" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -6039,7 +6039,7 @@
       </c>
       <c r="O95" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -6098,7 +6098,7 @@
       </c>
       <c r="O96" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -6157,7 +6157,7 @@
       </c>
       <c r="O97" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -6216,7 +6216,7 @@
       </c>
       <c r="O98" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -6275,7 +6275,7 @@
       </c>
       <c r="O99" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -6334,7 +6334,7 @@
       </c>
       <c r="O100" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -6393,7 +6393,7 @@
       </c>
       <c r="O101" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -6452,7 +6452,7 @@
       </c>
       <c r="O102" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -6511,7 +6511,7 @@
       </c>
       <c r="O103" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -6570,7 +6570,7 @@
       </c>
       <c r="O104" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -6629,7 +6629,7 @@
       </c>
       <c r="O105" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -6688,7 +6688,7 @@
       </c>
       <c r="O106" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -6747,7 +6747,7 @@
       </c>
       <c r="O107" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -6806,7 +6806,7 @@
       </c>
       <c r="O108" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -6865,7 +6865,7 @@
       </c>
       <c r="O109" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -6924,7 +6924,7 @@
       </c>
       <c r="O110" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -6983,7 +6983,7 @@
       </c>
       <c r="O111" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -7042,7 +7042,7 @@
       </c>
       <c r="O112" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -7101,7 +7101,7 @@
       </c>
       <c r="O113" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -7160,7 +7160,7 @@
       </c>
       <c r="O114" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -7219,7 +7219,7 @@
       </c>
       <c r="O115" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -7278,7 +7278,7 @@
       </c>
       <c r="O116" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -7337,7 +7337,7 @@
       </c>
       <c r="O117" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -7396,7 +7396,7 @@
       </c>
       <c r="O118" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -7455,7 +7455,7 @@
       </c>
       <c r="O119" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -7514,7 +7514,7 @@
       </c>
       <c r="O120" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -7573,7 +7573,7 @@
       </c>
       <c r="O121" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -7632,7 +7632,7 @@
       </c>
       <c r="O122" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -7691,7 +7691,7 @@
       </c>
       <c r="O123" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -7750,7 +7750,7 @@
       </c>
       <c r="O124" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -7809,7 +7809,7 @@
       </c>
       <c r="O125" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -7868,7 +7868,7 @@
       </c>
       <c r="O126" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -7927,7 +7927,7 @@
       </c>
       <c r="O127" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -7986,7 +7986,7 @@
       </c>
       <c r="O128" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -8045,7 +8045,7 @@
       </c>
       <c r="O129" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -8104,7 +8104,7 @@
       </c>
       <c r="O130" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -8163,7 +8163,7 @@
       </c>
       <c r="O131" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -8222,7 +8222,7 @@
       </c>
       <c r="O132" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -8281,7 +8281,7 @@
       </c>
       <c r="O133" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -8340,7 +8340,7 @@
       </c>
       <c r="O134" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -8399,7 +8399,7 @@
       </c>
       <c r="O135" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -8458,7 +8458,7 @@
       </c>
       <c r="O136" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -8517,7 +8517,7 @@
       </c>
       <c r="O137" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -8576,7 +8576,7 @@
       </c>
       <c r="O138" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -8635,7 +8635,7 @@
       </c>
       <c r="O139" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -8694,7 +8694,7 @@
       </c>
       <c r="O140" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -8753,7 +8753,7 @@
       </c>
       <c r="O141" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -8812,7 +8812,7 @@
       </c>
       <c r="O142" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -8871,7 +8871,7 @@
       </c>
       <c r="O143" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -8930,7 +8930,7 @@
       </c>
       <c r="O144" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -8989,7 +8989,7 @@
       </c>
       <c r="O145" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -9048,7 +9048,7 @@
       </c>
       <c r="O146" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -9107,7 +9107,7 @@
       </c>
       <c r="O147" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -9166,7 +9166,7 @@
       </c>
       <c r="O148" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -9225,7 +9225,7 @@
       </c>
       <c r="O149" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -9284,7 +9284,7 @@
       </c>
       <c r="O150" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -9343,7 +9343,7 @@
       </c>
       <c r="O151" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -9402,7 +9402,7 @@
       </c>
       <c r="O152" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -9461,7 +9461,7 @@
       </c>
       <c r="O153" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -9520,7 +9520,7 @@
       </c>
       <c r="O154" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -9579,7 +9579,7 @@
       </c>
       <c r="O155" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -9638,7 +9638,7 @@
       </c>
       <c r="O156" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -9697,7 +9697,7 @@
       </c>
       <c r="O157" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -9756,7 +9756,7 @@
       </c>
       <c r="O158" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -9815,7 +9815,7 @@
       </c>
       <c r="O159" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -9874,7 +9874,7 @@
       </c>
       <c r="O160" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -9933,7 +9933,7 @@
       </c>
       <c r="O161" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -9992,7 +9992,7 @@
       </c>
       <c r="O162" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -10051,7 +10051,7 @@
       </c>
       <c r="O163" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -10110,7 +10110,7 @@
       </c>
       <c r="O164" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -10169,7 +10169,7 @@
       </c>
       <c r="O165" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -10228,7 +10228,7 @@
       </c>
       <c r="O166" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -10287,7 +10287,7 @@
       </c>
       <c r="O167" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -10346,7 +10346,7 @@
       </c>
       <c r="O168" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -10405,7 +10405,7 @@
       </c>
       <c r="O169" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -10464,7 +10464,7 @@
       </c>
       <c r="O170" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -10523,7 +10523,7 @@
       </c>
       <c r="O171" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -10582,7 +10582,7 @@
       </c>
       <c r="O172" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -10641,7 +10641,7 @@
       </c>
       <c r="O173" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -10700,7 +10700,7 @@
       </c>
       <c r="O174" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -10759,7 +10759,7 @@
       </c>
       <c r="O175" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -10818,7 +10818,7 @@
       </c>
       <c r="O176" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -10877,7 +10877,7 @@
       </c>
       <c r="O177" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -10936,7 +10936,7 @@
       </c>
       <c r="O178" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -10995,7 +10995,7 @@
       </c>
       <c r="O179" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -11054,7 +11054,7 @@
       </c>
       <c r="O180" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -11113,7 +11113,7 @@
       </c>
       <c r="O181" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -11172,7 +11172,7 @@
       </c>
       <c r="O182" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -11231,7 +11231,7 @@
       </c>
       <c r="O183" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -11290,7 +11290,7 @@
       </c>
       <c r="O184" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -11349,7 +11349,7 @@
       </c>
       <c r="O185" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -11408,7 +11408,7 @@
       </c>
       <c r="O186" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -11467,7 +11467,7 @@
       </c>
       <c r="O187" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -11526,7 +11526,7 @@
       </c>
       <c r="O188" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -11585,7 +11585,7 @@
       </c>
       <c r="O189" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -11644,7 +11644,7 @@
       </c>
       <c r="O190" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -11703,7 +11703,7 @@
       </c>
       <c r="O191" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -11762,7 +11762,7 @@
       </c>
       <c r="O192" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -11821,7 +11821,7 @@
       </c>
       <c r="O193" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -11880,7 +11880,7 @@
       </c>
       <c r="O194" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -11939,7 +11939,7 @@
       </c>
       <c r="O195" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -11998,7 +11998,7 @@
       </c>
       <c r="O196" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -12057,7 +12057,7 @@
       </c>
       <c r="O197" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -12116,7 +12116,7 @@
       </c>
       <c r="O198" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -12175,7 +12175,7 @@
       </c>
       <c r="O199" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -12234,7 +12234,7 @@
       </c>
       <c r="O200" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -12293,7 +12293,7 @@
       </c>
       <c r="O201" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -12352,7 +12352,7 @@
       </c>
       <c r="O202" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -12411,7 +12411,7 @@
       </c>
       <c r="O203" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -12470,7 +12470,7 @@
       </c>
       <c r="O204" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -12529,7 +12529,7 @@
       </c>
       <c r="O205" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -12574,7 +12574,7 @@
       </c>
       <c r="O206" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -12633,7 +12633,7 @@
       </c>
       <c r="O207" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -12692,7 +12692,7 @@
       </c>
       <c r="O208" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -12751,7 +12751,7 @@
       </c>
       <c r="O209" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -12810,7 +12810,7 @@
       </c>
       <c r="O210" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -12869,7 +12869,7 @@
       </c>
       <c r="O211" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -12928,7 +12928,7 @@
       </c>
       <c r="O212" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -12987,7 +12987,7 @@
       </c>
       <c r="O213" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -13046,7 +13046,7 @@
       </c>
       <c r="O214" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -13105,7 +13105,7 @@
       </c>
       <c r="O215" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -13164,7 +13164,7 @@
       </c>
       <c r="O216" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -13223,7 +13223,7 @@
       </c>
       <c r="O217" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -13282,7 +13282,7 @@
       </c>
       <c r="O218" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -13341,7 +13341,7 @@
       </c>
       <c r="O219" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -13400,7 +13400,7 @@
       </c>
       <c r="O220" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -13459,7 +13459,7 @@
       </c>
       <c r="O221" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -13518,7 +13518,7 @@
       </c>
       <c r="O222" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -13577,7 +13577,7 @@
       </c>
       <c r="O223" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -13636,7 +13636,7 @@
       </c>
       <c r="O224" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -13695,7 +13695,7 @@
       </c>
       <c r="O225" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -13754,7 +13754,7 @@
       </c>
       <c r="O226" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -13813,7 +13813,7 @@
       </c>
       <c r="O227" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -13872,7 +13872,7 @@
       </c>
       <c r="O228" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -13931,7 +13931,7 @@
       </c>
       <c r="O229" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -13990,7 +13990,7 @@
       </c>
       <c r="O230" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -14049,7 +14049,7 @@
       </c>
       <c r="O231" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -14108,7 +14108,7 @@
       </c>
       <c r="O232" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -14167,7 +14167,7 @@
       </c>
       <c r="O233" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -14226,7 +14226,7 @@
       </c>
       <c r="O234" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -14285,7 +14285,7 @@
       </c>
       <c r="O235" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -14344,7 +14344,7 @@
       </c>
       <c r="O236" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -14403,7 +14403,7 @@
       </c>
       <c r="O237" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -14462,7 +14462,7 @@
       </c>
       <c r="O238" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -14521,7 +14521,7 @@
       </c>
       <c r="O239" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -14580,7 +14580,7 @@
       </c>
       <c r="O240" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -14639,7 +14639,7 @@
       </c>
       <c r="O241" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -14698,7 +14698,7 @@
       </c>
       <c r="O242" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -14757,7 +14757,7 @@
       </c>
       <c r="O243" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -14816,7 +14816,7 @@
       </c>
       <c r="O244" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -14875,7 +14875,7 @@
       </c>
       <c r="O245" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -14934,7 +14934,7 @@
       </c>
       <c r="O246" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -14993,7 +14993,7 @@
       </c>
       <c r="O247" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -15052,7 +15052,7 @@
       </c>
       <c r="O248" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -15111,7 +15111,7 @@
       </c>
       <c r="O249" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -15170,7 +15170,7 @@
       </c>
       <c r="O250" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -15229,7 +15229,7 @@
       </c>
       <c r="O251" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -15288,7 +15288,7 @@
       </c>
       <c r="O252" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -15347,7 +15347,7 @@
       </c>
       <c r="O253" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -15406,7 +15406,7 @@
       </c>
       <c r="O254" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -15465,7 +15465,7 @@
       </c>
       <c r="O255" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -15524,7 +15524,7 @@
       </c>
       <c r="O256" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -15583,7 +15583,7 @@
       </c>
       <c r="O257" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -15642,7 +15642,7 @@
       </c>
       <c r="O258" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -15701,7 +15701,7 @@
       </c>
       <c r="O259" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -15760,7 +15760,7 @@
       </c>
       <c r="O260" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -15819,7 +15819,7 @@
       </c>
       <c r="O261" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -15878,7 +15878,7 @@
       </c>
       <c r="O262" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -15937,7 +15937,7 @@
       </c>
       <c r="O263" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -15996,7 +15996,7 @@
       </c>
       <c r="O264" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -16055,7 +16055,7 @@
       </c>
       <c r="O265" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -16114,7 +16114,7 @@
       </c>
       <c r="O266" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -16173,7 +16173,7 @@
       </c>
       <c r="O267" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -16232,7 +16232,7 @@
       </c>
       <c r="O268" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -16291,7 +16291,7 @@
       </c>
       <c r="O269" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -16350,7 +16350,7 @@
       </c>
       <c r="O270" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -16409,7 +16409,7 @@
       </c>
       <c r="O271" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -16468,7 +16468,7 @@
       </c>
       <c r="O272" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -16527,7 +16527,7 @@
       </c>
       <c r="O273" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -16586,7 +16586,7 @@
       </c>
       <c r="O274" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -16645,7 +16645,7 @@
       </c>
       <c r="O275" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -16704,7 +16704,7 @@
       </c>
       <c r="O276" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -16763,7 +16763,7 @@
       </c>
       <c r="O277" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -16822,7 +16822,7 @@
       </c>
       <c r="O278" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -16881,7 +16881,7 @@
       </c>
       <c r="O279" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -16940,7 +16940,7 @@
       </c>
       <c r="O280" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -16999,7 +16999,7 @@
       </c>
       <c r="O281" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -17058,7 +17058,7 @@
       </c>
       <c r="O282" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -17117,7 +17117,7 @@
       </c>
       <c r="O283" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -17176,7 +17176,7 @@
       </c>
       <c r="O284" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -17235,7 +17235,7 @@
       </c>
       <c r="O285" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -17294,7 +17294,7 @@
       </c>
       <c r="O286" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -17353,7 +17353,7 @@
       </c>
       <c r="O287" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -17412,7 +17412,7 @@
       </c>
       <c r="O288" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -17471,7 +17471,7 @@
       </c>
       <c r="O289" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -17530,7 +17530,7 @@
       </c>
       <c r="O290" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -17589,7 +17589,7 @@
       </c>
       <c r="O291" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -17648,7 +17648,7 @@
       </c>
       <c r="O292" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -17707,7 +17707,7 @@
       </c>
       <c r="O293" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -17766,7 +17766,7 @@
       </c>
       <c r="O294" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -17825,7 +17825,7 @@
       </c>
       <c r="O295" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -17884,7 +17884,7 @@
       </c>
       <c r="O296" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -17943,7 +17943,7 @@
       </c>
       <c r="O297" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -18002,7 +18002,7 @@
       </c>
       <c r="O298" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -18061,7 +18061,7 @@
       </c>
       <c r="O299" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -18120,7 +18120,7 @@
       </c>
       <c r="O300" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -18179,7 +18179,7 @@
       </c>
       <c r="O301" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -18238,7 +18238,7 @@
       </c>
       <c r="O302" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -18297,7 +18297,7 @@
       </c>
       <c r="O303" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -18356,7 +18356,7 @@
       </c>
       <c r="O304" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -18415,7 +18415,7 @@
       </c>
       <c r="O305" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -18474,7 +18474,7 @@
       </c>
       <c r="O306" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -18533,7 +18533,7 @@
       </c>
       <c r="O307" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -18592,7 +18592,7 @@
       </c>
       <c r="O308" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -18651,7 +18651,7 @@
       </c>
       <c r="O309" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -18710,7 +18710,7 @@
       </c>
       <c r="O310" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -18769,7 +18769,7 @@
       </c>
       <c r="O311" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -18828,7 +18828,7 @@
       </c>
       <c r="O312" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -18887,7 +18887,7 @@
       </c>
       <c r="O313" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -18946,7 +18946,7 @@
       </c>
       <c r="O314" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -19005,7 +19005,7 @@
       </c>
       <c r="O315" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -19064,7 +19064,7 @@
       </c>
       <c r="O316" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -19123,7 +19123,7 @@
       </c>
       <c r="O317" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -19182,7 +19182,7 @@
       </c>
       <c r="O318" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -19241,7 +19241,7 @@
       </c>
       <c r="O319" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -19300,7 +19300,7 @@
       </c>
       <c r="O320" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -19359,7 +19359,7 @@
       </c>
       <c r="O321" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -19418,7 +19418,7 @@
       </c>
       <c r="O322" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -19477,7 +19477,7 @@
       </c>
       <c r="O323" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -19536,7 +19536,7 @@
       </c>
       <c r="O324" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -19595,7 +19595,7 @@
       </c>
       <c r="O325" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -19654,7 +19654,7 @@
       </c>
       <c r="O326" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -19713,7 +19713,7 @@
       </c>
       <c r="O327" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -19772,7 +19772,7 @@
       </c>
       <c r="O328" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -19831,7 +19831,7 @@
       </c>
       <c r="O329" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -19890,7 +19890,7 @@
       </c>
       <c r="O330" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -19949,7 +19949,7 @@
       </c>
       <c r="O331" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -20008,7 +20008,7 @@
       </c>
       <c r="O332" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -20067,7 +20067,7 @@
       </c>
       <c r="O333" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -20126,7 +20126,7 @@
       </c>
       <c r="O334" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -20185,7 +20185,7 @@
       </c>
       <c r="O335" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -20244,7 +20244,7 @@
       </c>
       <c r="O336" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -20303,7 +20303,7 @@
       </c>
       <c r="O337" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -20362,7 +20362,7 @@
       </c>
       <c r="O338" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -20407,7 +20407,7 @@
       </c>
       <c r="O339" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>
@@ -20466,7 +20466,7 @@
       </c>
       <c r="O340" t="inlineStr">
         <is>
-          <t>2026-10-28T09:49:28Z</t>
+          <t>2026-10-28T10:06:43Z</t>
         </is>
       </c>
     </row>

</xml_diff>